<commit_message>
xde agregando ingreso masivo para los 5 tipos de items
</commit_message>
<xml_diff>
--- a/src/data/FORMATO_SUBIDA_PRODUCTOS.xlsx
+++ b/src/data/FORMATO_SUBIDA_PRODUCTOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WebstormProjects\erpperu2-automation\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEDD12F6-0849-41E5-A55D-8ABD6A06E955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E0AC3A3-78E1-4E92-8113-FD087C6DE3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32220" yWindow="1470" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27270" yWindow="4260" windowWidth="21600" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCTOS" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PRODUCTOS!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -612,9 +617,6 @@
     <t>Krylon</t>
   </si>
   <si>
-    <t>ESTANDAR</t>
-  </si>
-  <si>
     <t>MAYORISTA</t>
   </si>
   <si>
@@ -772,6 +774,9 @@
   </si>
   <si>
     <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-6</t>
+  </si>
+  <si>
+    <t>PRECIO ESTÁNDAR</t>
   </si>
 </sst>
 </file>
@@ -1052,9 +1057,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1092,9 +1097,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1127,26 +1132,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1179,26 +1167,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1387,7 +1358,7 @@
     <col min="12" max="12" width="11.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="6" customFormat="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" s="6" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1413,21 +1384,21 @@
         <v>7</v>
       </c>
       <c r="I1" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="J1" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="K1" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="L1" s="14" t="s">
         <v>197</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B2" t="s">
         <v>113</v>
@@ -1465,7 +1436,7 @@
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B3" t="s">
         <v>116</v>
@@ -1503,7 +1474,7 @@
     </row>
     <row r="4" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B4" t="s">
         <v>116</v>
@@ -1541,7 +1512,7 @@
     </row>
     <row r="5" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B5" t="s">
         <v>119</v>
@@ -1579,7 +1550,7 @@
     </row>
     <row r="6" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B6" t="s">
         <v>122</v>
@@ -1617,7 +1588,7 @@
     </row>
     <row r="7" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B7" t="s">
         <v>125</v>
@@ -1655,7 +1626,7 @@
     </row>
     <row r="8" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B8" t="s">
         <v>127</v>
@@ -1693,7 +1664,7 @@
     </row>
     <row r="9" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B9" t="s">
         <v>129</v>
@@ -1731,7 +1702,7 @@
     </row>
     <row r="10" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B10" t="s">
         <v>131</v>
@@ -1769,7 +1740,7 @@
     </row>
     <row r="11" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B11" t="s">
         <v>134</v>
@@ -1807,7 +1778,7 @@
     </row>
     <row r="12" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B12" t="s">
         <v>136</v>
@@ -1845,7 +1816,7 @@
     </row>
     <row r="13" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B13" t="s">
         <v>138</v>
@@ -1883,7 +1854,7 @@
     </row>
     <row r="14" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B14" t="s">
         <v>141</v>
@@ -1921,7 +1892,7 @@
     </row>
     <row r="15" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B15" t="s">
         <v>142</v>
@@ -1959,7 +1930,7 @@
     </row>
     <row r="16" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B16" t="s">
         <v>145</v>
@@ -1997,7 +1968,7 @@
     </row>
     <row r="17" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B17" t="s">
         <v>147</v>
@@ -2035,7 +2006,7 @@
     </row>
     <row r="18" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B18" t="s">
         <v>149</v>
@@ -2073,7 +2044,7 @@
     </row>
     <row r="19" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B19" t="s">
         <v>151</v>
@@ -2111,7 +2082,7 @@
     </row>
     <row r="20" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B20" t="s">
         <v>154</v>
@@ -2149,7 +2120,7 @@
     </row>
     <row r="21" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B21" t="s">
         <v>141</v>
@@ -2187,7 +2158,7 @@
     </row>
     <row r="22" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B22" t="s">
         <v>157</v>
@@ -2225,7 +2196,7 @@
     </row>
     <row r="23" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B23" t="s">
         <v>158</v>
@@ -2263,7 +2234,7 @@
     </row>
     <row r="24" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B24" t="s">
         <v>113</v>
@@ -2301,7 +2272,7 @@
     </row>
     <row r="25" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B25" t="s">
         <v>161</v>
@@ -2339,7 +2310,7 @@
     </row>
     <row r="26" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B26" t="s">
         <v>162</v>
@@ -2377,7 +2348,7 @@
     </row>
     <row r="27" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B27" t="s">
         <v>163</v>
@@ -2415,7 +2386,7 @@
     </row>
     <row r="28" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B28" t="s">
         <v>164</v>
@@ -2453,7 +2424,7 @@
     </row>
     <row r="29" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B29" t="s">
         <v>167</v>
@@ -2491,7 +2462,7 @@
     </row>
     <row r="30" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B30" t="s">
         <v>168</v>
@@ -2529,7 +2500,7 @@
     </row>
     <row r="31" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B31" t="s">
         <v>171</v>
@@ -2567,7 +2538,7 @@
     </row>
     <row r="32" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B32" t="s">
         <v>172</v>
@@ -2605,7 +2576,7 @@
     </row>
     <row r="33" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B33" t="s">
         <v>175</v>
@@ -2643,7 +2614,7 @@
     </row>
     <row r="34" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B34" t="s">
         <v>176</v>
@@ -2681,7 +2652,7 @@
     </row>
     <row r="35" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B35" t="s">
         <v>179</v>
@@ -2719,7 +2690,7 @@
     </row>
     <row r="36" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B36" t="s">
         <v>180</v>
@@ -2757,7 +2728,7 @@
     </row>
     <row r="37" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B37" t="s">
         <v>181</v>
@@ -2795,7 +2766,7 @@
     </row>
     <row r="38" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B38" t="s">
         <v>181</v>
@@ -2833,7 +2804,7 @@
     </row>
     <row r="39" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B39" t="s">
         <v>172</v>
@@ -2871,7 +2842,7 @@
     </row>
     <row r="40" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B40" t="s">
         <v>185</v>
@@ -2909,7 +2880,7 @@
     </row>
     <row r="41" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B41" t="s">
         <v>113</v>
@@ -2947,7 +2918,7 @@
     </row>
     <row r="42" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B42" t="s">
         <v>113</v>
@@ -2985,7 +2956,7 @@
     </row>
     <row r="43" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B43" t="s">
         <v>188</v>
@@ -3023,7 +2994,7 @@
     </row>
     <row r="44" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B44" t="s">
         <v>189</v>
@@ -3061,7 +3032,7 @@
     </row>
     <row r="45" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B45" t="s">
         <v>190</v>
@@ -3099,7 +3070,7 @@
     </row>
     <row r="46" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B46" t="s">
         <v>141</v>
@@ -3137,7 +3108,7 @@
     </row>
     <row r="47" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B47" t="s">
         <v>190</v>
@@ -3175,7 +3146,7 @@
     </row>
     <row r="48" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B48" t="s">
         <v>191</v>
@@ -3213,7 +3184,7 @@
     </row>
     <row r="49" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B49" t="s">
         <v>192</v>
@@ -3251,7 +3222,7 @@
     </row>
     <row r="50" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B50" t="s">
         <v>193</v>
@@ -3289,7 +3260,7 @@
     </row>
     <row r="51" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B51" t="s">
         <v>194</v>

</xml_diff>

<commit_message>
⚡Fix intentos de test
</commit_message>
<xml_diff>
--- a/src/data/FORMATO_SUBIDA_PRODUCTOS.xlsx
+++ b/src/data/FORMATO_SUBIDA_PRODUCTOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WebstormProjects\erpperu2-automation\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E0AC3A3-78E1-4E92-8113-FD087C6DE3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B6BA12-DD08-4B1D-B6C6-BA08DEF66E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27270" yWindow="4260" windowWidth="21600" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCTOS" sheetId="1" r:id="rId1"/>
@@ -30,753 +30,576 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="190">
+  <si>
+    <t>MARCA</t>
+  </si>
+  <si>
+    <t>CATEGORIA</t>
+  </si>
+  <si>
+    <t>SUB CATEGORIA</t>
+  </si>
+  <si>
+    <t>SIN CONTROL DE STOCK</t>
+  </si>
+  <si>
+    <t>CONTROL DE STOCK ESTRICTO</t>
+  </si>
+  <si>
+    <t>CONTROL DE STOCK FLEXIBLE</t>
+  </si>
+  <si>
+    <t>TIPO AFECTACION IGV</t>
+  </si>
+  <si>
+    <t>CLASE</t>
+  </si>
+  <si>
+    <t>BIEN</t>
+  </si>
+  <si>
+    <t>SERVICIO</t>
+  </si>
+  <si>
+    <t>USO</t>
+  </si>
+  <si>
+    <t>COMPRA Y VENTA</t>
+  </si>
+  <si>
+    <t>COMPRA</t>
+  </si>
+  <si>
+    <t>VENTA</t>
+  </si>
+  <si>
+    <t>VALORIZACIÓN</t>
+  </si>
+  <si>
+    <t>FIFO</t>
+  </si>
+  <si>
+    <t>PROMEDIO</t>
+  </si>
+  <si>
+    <t>RESPUESTA</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>ESTADO</t>
+  </si>
+  <si>
+    <t>ACTIVO</t>
+  </si>
+  <si>
+    <t>TIPOPRECIOUNITARIO</t>
+  </si>
+  <si>
+    <t>PRECIO UNITARIO (VENTAS)</t>
+  </si>
+  <si>
+    <t>PRODUCTO PARA REGALO O BONIFICACION</t>
+  </si>
+  <si>
+    <t>TIPOAFECTACIONIGV</t>
+  </si>
+  <si>
+    <t>GRAVADO - PAGA IGV</t>
+  </si>
+  <si>
+    <t>GRAVADO - RETIRO POR PREMIO</t>
+  </si>
+  <si>
+    <t>GRAVADO - RETIRO POR DONACION</t>
+  </si>
+  <si>
+    <t>GRAVADO - RETIRO</t>
+  </si>
+  <si>
+    <t>GRAVADO - RETIRO POR PUBLICIDAD</t>
+  </si>
+  <si>
+    <t>GRAVADO - BONIFICACIONES</t>
+  </si>
+  <si>
+    <t>GRAVADO - RETIRO POR ENTREGA A TRABAJADORES</t>
+  </si>
+  <si>
+    <t>EXONERADO - NO PAGA IGV</t>
+  </si>
+  <si>
+    <t>EXONERADO - TRANSFERENCIA GRATUITA</t>
+  </si>
+  <si>
+    <t>INAFECTO - NO PAGA IGV</t>
+  </si>
+  <si>
+    <t>INAFECTO - RETIRO POR BONIFICACION</t>
+  </si>
+  <si>
+    <t>INAFECTO - RETIRO</t>
+  </si>
+  <si>
+    <t>INAFECTO - RETIRO POR MUESTRAS MEDICAS</t>
+  </si>
+  <si>
+    <t>INAFECTO - RETIRO POR CONVENIO COLECTIVO</t>
+  </si>
+  <si>
+    <t>INAFECTO - RETIRO POR PREMIO</t>
+  </si>
+  <si>
+    <t>INAFECTO - RETIRO POR PUBLICIDAD</t>
+  </si>
+  <si>
+    <t>TIPOCODIGODEBARRAS</t>
+  </si>
+  <si>
+    <t>PROPIO</t>
+  </si>
+  <si>
+    <t>GTIN-8</t>
+  </si>
+  <si>
+    <t>GTIN-12</t>
+  </si>
+  <si>
+    <t>GTIN-13</t>
+  </si>
+  <si>
+    <t>GTIN-14</t>
+  </si>
+  <si>
+    <t>UNIDADES EQUIVALENTE SUNAT</t>
+  </si>
+  <si>
+    <t>Bobbin</t>
+  </si>
+  <si>
+    <t>bucket</t>
+  </si>
+  <si>
+    <t>barrel (US) (petroleum etc.)</t>
+  </si>
+  <si>
+    <t>bag</t>
+  </si>
+  <si>
+    <t>bottle</t>
+  </si>
+  <si>
+    <t>Box</t>
+  </si>
+  <si>
+    <t>Carton</t>
+  </si>
+  <si>
+    <t>square centimetre</t>
+  </si>
+  <si>
+    <t>cubic centimeter</t>
+  </si>
+  <si>
+    <t>Centimeter</t>
+  </si>
+  <si>
+    <t>Hundred</t>
+  </si>
+  <si>
+    <t>cylinder</t>
+  </si>
+  <si>
+    <t>Cone</t>
+  </si>
+  <si>
+    <t>Dozen</t>
+  </si>
+  <si>
+    <t>dozen pack</t>
+  </si>
+  <si>
+    <t>bundle</t>
+  </si>
+  <si>
+    <t>number of international units</t>
+  </si>
+  <si>
+    <t>ton (US) or short ton (UK/US)</t>
+  </si>
+  <si>
+    <t>ton (UK) or longton (US)</t>
+  </si>
+  <si>
+    <t>package</t>
+  </si>
+  <si>
+    <t>Foot</t>
+  </si>
+  <si>
+    <t>square foot</t>
+  </si>
+  <si>
+    <t>Can</t>
+  </si>
+  <si>
+    <t>Litre</t>
+  </si>
+  <si>
+    <t>cubic foot</t>
+  </si>
+  <si>
+    <t>metre</t>
+  </si>
+  <si>
+    <t>square metre</t>
+  </si>
+  <si>
+    <t>cubic metre</t>
+  </si>
+  <si>
+    <t>kilogram</t>
+  </si>
+  <si>
+    <t>ounce</t>
+  </si>
+  <si>
+    <t>US GALON (3,7843 L)</t>
+  </si>
+  <si>
+    <t>GRAM</t>
+  </si>
+  <si>
+    <t>POUND</t>
+  </si>
+  <si>
+    <t>MILLILITRE</t>
+  </si>
+  <si>
+    <t>TIN</t>
+  </si>
+  <si>
+    <t>MILLE</t>
+  </si>
+  <si>
+    <t>SET</t>
+  </si>
+  <si>
+    <t>KILOAMPERE</t>
+  </si>
+  <si>
+    <t>KILOBYTE</t>
+  </si>
+  <si>
+    <t>JUEGO</t>
+  </si>
+  <si>
+    <t>PAR</t>
+  </si>
+  <si>
+    <t>KIT</t>
+  </si>
+  <si>
+    <t>HOJA</t>
+  </si>
+  <si>
+    <t>PALETAS</t>
+  </si>
+  <si>
+    <t>MILIGRAMOS</t>
+  </si>
+  <si>
+    <t>PIEZA</t>
+  </si>
+  <si>
+    <t>RESMA</t>
+  </si>
+  <si>
+    <t>KILOMETRO</t>
+  </si>
+  <si>
+    <t>MILIMETRO</t>
+  </si>
+  <si>
+    <t>MILIMETRO CUADRADO</t>
+  </si>
+  <si>
+    <t>MILIMETRO CUBICO</t>
+  </si>
+  <si>
+    <t>MILLON DE UNIDADES</t>
+  </si>
+  <si>
+    <t>PLIEGO</t>
+  </si>
+  <si>
+    <t>PULGADAS</t>
+  </si>
+  <si>
+    <t>TONELADAS</t>
+  </si>
+  <si>
+    <t>TUBOS</t>
+  </si>
+  <si>
+    <t>UNIDAD (SERVICIOS)</t>
+  </si>
+  <si>
+    <t>YARDA</t>
+  </si>
+  <si>
+    <t>MILLARES</t>
+  </si>
+  <si>
+    <t>GRUESA</t>
+  </si>
+  <si>
+    <t>GALON INGLES</t>
+  </si>
+  <si>
+    <t>TAMBOR</t>
+  </si>
+  <si>
+    <t>TIPOAFECTACIONIGV SIMPLE</t>
+  </si>
+  <si>
+    <t>Truper</t>
+  </si>
+  <si>
+    <t>Herramientas</t>
+  </si>
+  <si>
+    <t>Manuales</t>
+  </si>
+  <si>
+    <t>Bosch</t>
+  </si>
+  <si>
+    <t>Eléctricas</t>
+  </si>
+  <si>
+    <t>Medición y Trazo</t>
+  </si>
+  <si>
+    <t>Norton</t>
+  </si>
+  <si>
+    <t>Accesorios</t>
+  </si>
+  <si>
+    <t>Abrasivos y Brocas</t>
+  </si>
+  <si>
+    <t>Hilti</t>
+  </si>
+  <si>
+    <t>Tornillería</t>
+  </si>
+  <si>
+    <t>Anclajes y Fijaciones</t>
+  </si>
+  <si>
+    <t>Simpson Strong-Tie</t>
+  </si>
+  <si>
+    <t>Tornillos para Madera</t>
+  </si>
+  <si>
+    <t>Red Head</t>
+  </si>
+  <si>
+    <t>Anclajes Mecánicos</t>
+  </si>
+  <si>
+    <t>Fischer</t>
+  </si>
+  <si>
+    <t>Anclajes Químicos</t>
+  </si>
+  <si>
+    <t>Tigre</t>
+  </si>
+  <si>
+    <t>Plomería</t>
+  </si>
+  <si>
+    <t>PVC y CPVC</t>
+  </si>
+  <si>
+    <t>Mueller</t>
+  </si>
+  <si>
+    <t>Cobre y Gas</t>
+  </si>
+  <si>
+    <t>Helvex</t>
+  </si>
+  <si>
+    <t>Grifería y Válvulas</t>
+  </si>
+  <si>
+    <t>Sika</t>
+  </si>
+  <si>
+    <t>Químicos</t>
+  </si>
+  <si>
+    <t>Adhesivos y Selladores</t>
+  </si>
+  <si>
+    <t>3M</t>
+  </si>
+  <si>
+    <t>Indeco</t>
+  </si>
+  <si>
+    <t>Electricidad</t>
+  </si>
+  <si>
+    <t>Cables THHN/THW</t>
+  </si>
+  <si>
+    <t>Schneider Electric</t>
+  </si>
+  <si>
+    <t>Protección y Tableros</t>
+  </si>
+  <si>
+    <t>Philips</t>
+  </si>
+  <si>
+    <t>Iluminación</t>
+  </si>
+  <si>
+    <t>Legrand</t>
+  </si>
+  <si>
+    <t>Instalación y Accesorios</t>
+  </si>
+  <si>
+    <t>Comex</t>
+  </si>
+  <si>
+    <t>Pinturas y Acabados</t>
+  </si>
+  <si>
+    <t>Pinturas y Accesorios</t>
+  </si>
+  <si>
+    <t>Sayer</t>
+  </si>
+  <si>
+    <t>Seguridad</t>
+  </si>
+  <si>
+    <t>Equipo de Protección Personal</t>
+  </si>
+  <si>
+    <t>MSA</t>
+  </si>
+  <si>
+    <t>Ansell</t>
+  </si>
+  <si>
+    <t>Jardinería y Riego</t>
+  </si>
+  <si>
+    <t>Riego y Lavado</t>
+  </si>
+  <si>
+    <t>Gardena</t>
+  </si>
+  <si>
+    <t>MAYORISTA</t>
+  </si>
+  <si>
+    <t>DOLARES</t>
+  </si>
+  <si>
+    <t>COSTO</t>
+  </si>
+  <si>
+    <t>Llave ajustable 10" estricto gravado-1</t>
+  </si>
+  <si>
+    <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-2</t>
+  </si>
+  <si>
+    <t>Nivel láser GLL 2-15 estricto gravado-3</t>
+  </si>
+  <si>
+    <t>Disco flap 4-1/2" grano 60 estricto gravado-4</t>
+  </si>
+  <si>
+    <t>Llave ajustable 10" estricto gravado-2</t>
+  </si>
+  <si>
+    <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-3</t>
+  </si>
+  <si>
+    <t>Nivel láser GLL 2-15 estricto gravado-4</t>
+  </si>
+  <si>
+    <t>Disco flap 4-1/2" grano 60 estricto gravado-5</t>
+  </si>
+  <si>
+    <t>Tornillo para concreto HUS3 M8 x 100 estricto gravado-5</t>
+  </si>
+  <si>
+    <t>Tornillo estructural para madera 8 x 2" estricto exonerado-6</t>
+  </si>
+  <si>
+    <t>Anclaje wedge Trubolt 5/8" x 6" estricto exonerado-7</t>
+  </si>
+  <si>
+    <t>Cartucho resina FIS V 300 ml estricto exonerado-8</t>
+  </si>
+  <si>
+    <t>Tubo PVC hidráulico 25 mm 6 m estricto exonerado-9</t>
+  </si>
+  <si>
+    <t>Tubería de cobre tipo L 3/4" estricto exonerado-10</t>
+  </si>
+  <si>
+    <t>Mezcladora lavabo monomando estricto inafecto-11</t>
+  </si>
+  <si>
+    <t>SikaTop Seal 5 impermeabilizante 4kg estricto inafecto-12</t>
+  </si>
+  <si>
+    <t>Tornillo para concreto HUS3 M8 x 100 estricto gravado-6</t>
+  </si>
+  <si>
+    <t>Tornillo estructural para madera 8 x 2" estricto exonerado-7</t>
+  </si>
+  <si>
+    <t>PRECIO ESTÁNDAR</t>
+  </si>
   <si>
     <t>DESCRIPCION</t>
   </si>
   <si>
-    <t>MARCA</t>
-  </si>
-  <si>
-    <t>CATEGORIA</t>
-  </si>
-  <si>
-    <t>SUB CATEGORIA</t>
-  </si>
-  <si>
-    <t>SIN CONTROL DE STOCK</t>
-  </si>
-  <si>
-    <t>CONTROL DE STOCK ESTRICTO</t>
-  </si>
-  <si>
-    <t>CONTROL DE STOCK FLEXIBLE</t>
-  </si>
-  <si>
-    <t>TIPO AFECTACION IGV</t>
-  </si>
-  <si>
-    <t>CLASE</t>
-  </si>
-  <si>
-    <t>BIEN</t>
-  </si>
-  <si>
-    <t>SERVICIO</t>
-  </si>
-  <si>
-    <t>USO</t>
-  </si>
-  <si>
-    <t>COMPRA Y VENTA</t>
-  </si>
-  <si>
-    <t>COMPRA</t>
-  </si>
-  <si>
-    <t>VENTA</t>
-  </si>
-  <si>
-    <t>VALORIZACIÓN</t>
-  </si>
-  <si>
-    <t>FIFO</t>
-  </si>
-  <si>
-    <t>PROMEDIO</t>
-  </si>
-  <si>
-    <t>RESPUESTA</t>
-  </si>
-  <si>
-    <t>SI</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>ESTADO</t>
-  </si>
-  <si>
-    <t>ACTIVO</t>
-  </si>
-  <si>
-    <t>TIPOPRECIOUNITARIO</t>
-  </si>
-  <si>
-    <t>PRECIO UNITARIO (VENTAS)</t>
-  </si>
-  <si>
-    <t>PRODUCTO PARA REGALO O BONIFICACION</t>
-  </si>
-  <si>
-    <t>TIPOAFECTACIONIGV</t>
-  </si>
-  <si>
-    <t>GRAVADO - PAGA IGV</t>
-  </si>
-  <si>
-    <t>GRAVADO - RETIRO POR PREMIO</t>
-  </si>
-  <si>
-    <t>GRAVADO - RETIRO POR DONACION</t>
-  </si>
-  <si>
-    <t>GRAVADO - RETIRO</t>
-  </si>
-  <si>
-    <t>GRAVADO - RETIRO POR PUBLICIDAD</t>
-  </si>
-  <si>
-    <t>GRAVADO - BONIFICACIONES</t>
-  </si>
-  <si>
-    <t>GRAVADO - RETIRO POR ENTREGA A TRABAJADORES</t>
-  </si>
-  <si>
-    <t>EXONERADO - NO PAGA IGV</t>
-  </si>
-  <si>
-    <t>EXONERADO - TRANSFERENCIA GRATUITA</t>
-  </si>
-  <si>
-    <t>INAFECTO - NO PAGA IGV</t>
-  </si>
-  <si>
-    <t>INAFECTO - RETIRO POR BONIFICACION</t>
-  </si>
-  <si>
-    <t>INAFECTO - RETIRO</t>
-  </si>
-  <si>
-    <t>INAFECTO - RETIRO POR MUESTRAS MEDICAS</t>
-  </si>
-  <si>
-    <t>INAFECTO - RETIRO POR CONVENIO COLECTIVO</t>
-  </si>
-  <si>
-    <t>INAFECTO - RETIRO POR PREMIO</t>
-  </si>
-  <si>
-    <t>INAFECTO - RETIRO POR PUBLICIDAD</t>
-  </si>
-  <si>
-    <t>TIPOCODIGODEBARRAS</t>
-  </si>
-  <si>
-    <t>PROPIO</t>
-  </si>
-  <si>
-    <t>GTIN-8</t>
-  </si>
-  <si>
-    <t>GTIN-12</t>
-  </si>
-  <si>
-    <t>GTIN-13</t>
-  </si>
-  <si>
-    <t>GTIN-14</t>
-  </si>
-  <si>
-    <t>UNIDADES EQUIVALENTE SUNAT</t>
-  </si>
-  <si>
-    <t>Bobbin</t>
-  </si>
-  <si>
-    <t>bucket</t>
-  </si>
-  <si>
-    <t>barrel (US) (petroleum etc.)</t>
-  </si>
-  <si>
-    <t>bag</t>
-  </si>
-  <si>
-    <t>bottle</t>
-  </si>
-  <si>
-    <t>Box</t>
-  </si>
-  <si>
-    <t>Carton</t>
-  </si>
-  <si>
-    <t>square centimetre</t>
-  </si>
-  <si>
-    <t>cubic centimeter</t>
-  </si>
-  <si>
-    <t>Centimeter</t>
-  </si>
-  <si>
-    <t>Hundred</t>
-  </si>
-  <si>
-    <t>cylinder</t>
-  </si>
-  <si>
-    <t>Cone</t>
-  </si>
-  <si>
-    <t>Dozen</t>
-  </si>
-  <si>
-    <t>dozen pack</t>
-  </si>
-  <si>
-    <t>bundle</t>
-  </si>
-  <si>
-    <t>number of international units</t>
-  </si>
-  <si>
-    <t>ton (US) or short ton (UK/US)</t>
-  </si>
-  <si>
-    <t>ton (UK) or longton (US)</t>
-  </si>
-  <si>
-    <t>package</t>
-  </si>
-  <si>
-    <t>Foot</t>
-  </si>
-  <si>
-    <t>square foot</t>
-  </si>
-  <si>
-    <t>Can</t>
-  </si>
-  <si>
-    <t>Litre</t>
-  </si>
-  <si>
-    <t>cubic foot</t>
-  </si>
-  <si>
-    <t>metre</t>
-  </si>
-  <si>
-    <t>square metre</t>
-  </si>
-  <si>
-    <t>cubic metre</t>
-  </si>
-  <si>
-    <t>kilogram</t>
-  </si>
-  <si>
-    <t>ounce</t>
-  </si>
-  <si>
-    <t>US GALON (3,7843 L)</t>
-  </si>
-  <si>
-    <t>GRAM</t>
-  </si>
-  <si>
-    <t>POUND</t>
-  </si>
-  <si>
-    <t>MILLILITRE</t>
-  </si>
-  <si>
-    <t>TIN</t>
-  </si>
-  <si>
-    <t>MILLE</t>
-  </si>
-  <si>
-    <t>SET</t>
-  </si>
-  <si>
-    <t>KILOAMPERE</t>
-  </si>
-  <si>
-    <t>KILOBYTE</t>
-  </si>
-  <si>
-    <t>JUEGO</t>
-  </si>
-  <si>
-    <t>PAR</t>
-  </si>
-  <si>
-    <t>KIT</t>
-  </si>
-  <si>
-    <t>HOJA</t>
-  </si>
-  <si>
-    <t>PALETAS</t>
-  </si>
-  <si>
-    <t>MILIGRAMOS</t>
-  </si>
-  <si>
-    <t>PIEZA</t>
-  </si>
-  <si>
-    <t>RESMA</t>
-  </si>
-  <si>
-    <t>KILOMETRO</t>
-  </si>
-  <si>
-    <t>MILIMETRO</t>
-  </si>
-  <si>
-    <t>MILIMETRO CUADRADO</t>
-  </si>
-  <si>
-    <t>MILIMETRO CUBICO</t>
-  </si>
-  <si>
-    <t>MILLON DE UNIDADES</t>
-  </si>
-  <si>
-    <t>PLIEGO</t>
-  </si>
-  <si>
-    <t>PULGADAS</t>
-  </si>
-  <si>
-    <t>TONELADAS</t>
-  </si>
-  <si>
-    <t>TUBOS</t>
-  </si>
-  <si>
-    <t>UNIDAD (SERVICIOS)</t>
-  </si>
-  <si>
-    <t>YARDA</t>
-  </si>
-  <si>
-    <t>MILLARES</t>
-  </si>
-  <si>
-    <t>GRUESA</t>
-  </si>
-  <si>
-    <t>GALON INGLES</t>
-  </si>
-  <si>
-    <t>TAMBOR</t>
-  </si>
-  <si>
-    <t>TIPOAFECTACIONIGV SIMPLE</t>
-  </si>
-  <si>
-    <t>Truper</t>
-  </si>
-  <si>
-    <t>Herramientas</t>
-  </si>
-  <si>
-    <t>Manuales</t>
-  </si>
-  <si>
-    <t>Bosch</t>
-  </si>
-  <si>
-    <t>Eléctricas</t>
-  </si>
-  <si>
-    <t>Medición y Trazo</t>
-  </si>
-  <si>
-    <t>Norton</t>
-  </si>
-  <si>
-    <t>Accesorios</t>
-  </si>
-  <si>
-    <t>Abrasivos y Brocas</t>
-  </si>
-  <si>
-    <t>Hilti</t>
-  </si>
-  <si>
-    <t>Tornillería</t>
-  </si>
-  <si>
-    <t>Anclajes y Fijaciones</t>
-  </si>
-  <si>
-    <t>Simpson Strong-Tie</t>
-  </si>
-  <si>
-    <t>Tornillos para Madera</t>
-  </si>
-  <si>
-    <t>Red Head</t>
-  </si>
-  <si>
-    <t>Anclajes Mecánicos</t>
-  </si>
-  <si>
-    <t>Fischer</t>
-  </si>
-  <si>
-    <t>Anclajes Químicos</t>
-  </si>
-  <si>
-    <t>Tigre</t>
-  </si>
-  <si>
-    <t>Plomería</t>
-  </si>
-  <si>
-    <t>PVC y CPVC</t>
-  </si>
-  <si>
-    <t>Mueller</t>
-  </si>
-  <si>
-    <t>Cobre y Gas</t>
-  </si>
-  <si>
-    <t>Helvex</t>
-  </si>
-  <si>
-    <t>Grifería y Válvulas</t>
-  </si>
-  <si>
-    <t>Sika</t>
-  </si>
-  <si>
-    <t>Químicos</t>
-  </si>
-  <si>
-    <t>Adhesivos y Selladores</t>
-  </si>
-  <si>
-    <t>3M</t>
-  </si>
-  <si>
-    <t>Indeco</t>
-  </si>
-  <si>
-    <t>Electricidad</t>
-  </si>
-  <si>
-    <t>Cables THHN/THW</t>
-  </si>
-  <si>
-    <t>Schneider Electric</t>
-  </si>
-  <si>
-    <t>Protección y Tableros</t>
-  </si>
-  <si>
-    <t>Philips</t>
-  </si>
-  <si>
-    <t>Iluminación</t>
-  </si>
-  <si>
-    <t>Legrand</t>
-  </si>
-  <si>
-    <t>Instalación y Accesorios</t>
-  </si>
-  <si>
-    <t>Comex</t>
-  </si>
-  <si>
-    <t>Pinturas y Acabados</t>
-  </si>
-  <si>
-    <t>Pinturas y Accesorios</t>
-  </si>
-  <si>
-    <t>Sayer</t>
-  </si>
-  <si>
-    <t>Seguridad</t>
-  </si>
-  <si>
-    <t>Equipo de Protección Personal</t>
-  </si>
-  <si>
-    <t>MSA</t>
-  </si>
-  <si>
-    <t>Ansell</t>
-  </si>
-  <si>
-    <t>Jardinería y Riego</t>
-  </si>
-  <si>
-    <t>Riego y Lavado</t>
-  </si>
-  <si>
-    <t>Gardena</t>
-  </si>
-  <si>
-    <t>Karcher</t>
-  </si>
-  <si>
-    <t>Hunter</t>
-  </si>
-  <si>
-    <t>Werner</t>
-  </si>
-  <si>
-    <t>Acceso</t>
-  </si>
-  <si>
-    <t>Escaleras y Andamios</t>
-  </si>
-  <si>
-    <t>Louisville</t>
-  </si>
-  <si>
-    <t>Miller</t>
-  </si>
-  <si>
-    <t>Soldadura y Corte</t>
-  </si>
-  <si>
-    <t>Equipos y Consumibles</t>
-  </si>
-  <si>
-    <t>Harris</t>
-  </si>
-  <si>
-    <t>Stanley</t>
-  </si>
-  <si>
-    <t>Aire y Neumática</t>
-  </si>
-  <si>
-    <t>Compresores y Accesorios</t>
-  </si>
-  <si>
-    <t>Parker</t>
-  </si>
-  <si>
-    <t>Yale</t>
-  </si>
-  <si>
-    <t>Ferretería General</t>
-  </si>
-  <si>
-    <t>Cerraduras y Candados</t>
-  </si>
-  <si>
-    <t>Phillips</t>
-  </si>
-  <si>
-    <t>Abus</t>
-  </si>
-  <si>
-    <t>Blum</t>
-  </si>
-  <si>
-    <t>Herrajes para Mueble</t>
-  </si>
-  <si>
-    <t>Organización</t>
-  </si>
-  <si>
-    <t>Almacenaje y Cajas</t>
-  </si>
-  <si>
-    <t>Keter</t>
-  </si>
-  <si>
-    <t>Movimiento de Carga</t>
-  </si>
-  <si>
-    <t>Carretillas y Diablos</t>
-  </si>
-  <si>
-    <t>LEDVANCE</t>
-  </si>
-  <si>
-    <t>Sylvania</t>
-  </si>
-  <si>
-    <t>Osram</t>
-  </si>
-  <si>
-    <t>Bellota</t>
-  </si>
-  <si>
-    <t>Makita</t>
-  </si>
-  <si>
-    <t>DeWalt</t>
-  </si>
-  <si>
-    <t>Krylon</t>
-  </si>
-  <si>
-    <t>MAYORISTA</t>
-  </si>
-  <si>
-    <t>DOLARES</t>
-  </si>
-  <si>
-    <t>COSTO</t>
-  </si>
-  <si>
-    <t>Llave ajustable 10" estricto gravado-1</t>
-  </si>
-  <si>
-    <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-2</t>
-  </si>
-  <si>
-    <t>Nivel láser GLL 2-15 estricto gravado-3</t>
-  </si>
-  <si>
-    <t>Disco flap 4-1/2" grano 60 estricto gravado-4</t>
-  </si>
-  <si>
-    <t>Llave ajustable 10" estricto gravado-2</t>
-  </si>
-  <si>
-    <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-3</t>
-  </si>
-  <si>
-    <t>Nivel láser GLL 2-15 estricto gravado-4</t>
-  </si>
-  <si>
-    <t>Disco flap 4-1/2" grano 60 estricto gravado-5</t>
-  </si>
-  <si>
-    <t>Llave ajustable 10" estricto gravado-3</t>
-  </si>
-  <si>
-    <t>Tornillo para concreto HUS3 M8 x 100 estricto gravado-5</t>
-  </si>
-  <si>
-    <t>Tornillo estructural para madera 8 x 2" estricto exonerado-6</t>
-  </si>
-  <si>
-    <t>Anclaje wedge Trubolt 5/8" x 6" estricto exonerado-7</t>
-  </si>
-  <si>
-    <t>Cartucho resina FIS V 300 ml estricto exonerado-8</t>
-  </si>
-  <si>
-    <t>Tubo PVC hidráulico 25 mm 6 m estricto exonerado-9</t>
-  </si>
-  <si>
-    <t>Tubería de cobre tipo L 3/4" estricto exonerado-10</t>
-  </si>
-  <si>
-    <t>Mezcladora lavabo monomando estricto inafecto-11</t>
-  </si>
-  <si>
-    <t>SikaTop Seal 5 impermeabilizante 4kg estricto inafecto-12</t>
-  </si>
-  <si>
-    <t>Tornillo para concreto HUS3 M8 x 100 estricto gravado-6</t>
-  </si>
-  <si>
-    <t>Tornillo estructural para madera 8 x 2" estricto exonerado-7</t>
-  </si>
-  <si>
-    <t>Anclaje wedge Trubolt 5/8" x 6" estricto exonerado-8</t>
-  </si>
-  <si>
-    <t>Cartucho resina FIS V 300 ml estricto exonerado-9</t>
-  </si>
-  <si>
-    <t>Tubo PVC hidráulico 25 mm 6 m estricto exonerado-10</t>
-  </si>
-  <si>
-    <t>Tubería de cobre tipo L 3/4" estricto exonerado-11</t>
-  </si>
-  <si>
-    <t>Mezcladora lavabo monomando estricto inafecto-12</t>
-  </si>
-  <si>
-    <t>SikaTop Seal 5 impermeabilizante 4kg estricto inafecto-13</t>
-  </si>
-  <si>
-    <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-4</t>
-  </si>
-  <si>
-    <t>Nivel láser GLL 2-15 estricto gravado-5</t>
-  </si>
-  <si>
-    <t>Disco flap 4-1/2" grano 60 estricto gravado-6</t>
-  </si>
-  <si>
-    <t>Tornillo para concreto HUS3 M8 x 100 estricto gravado-7</t>
-  </si>
-  <si>
-    <t>Tornillo estructural para madera 8 x 2" estricto exonerado-8</t>
-  </si>
-  <si>
-    <t>Anclaje wedge Trubolt 5/8" x 6" estricto exonerado-9</t>
-  </si>
-  <si>
-    <t>Cartucho resina FIS V 300 ml estricto exonerado-10</t>
-  </si>
-  <si>
-    <t>Tubo PVC hidráulico 25 mm 6 m estricto exonerado-11</t>
-  </si>
-  <si>
-    <t>Tubería de cobre tipo L 3/4" estricto exonerado-12</t>
-  </si>
-  <si>
-    <t>Mezcladora lavabo monomando estricto inafecto-13</t>
-  </si>
-  <si>
-    <t>SikaTop Seal 5 impermeabilizante 4kg estricto inafecto-14</t>
-  </si>
-  <si>
-    <t>Llave ajustable 10" estricto gravado-4</t>
-  </si>
-  <si>
-    <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-5</t>
-  </si>
-  <si>
-    <t>Nivel láser GLL 2-15 estricto gravado-6</t>
-  </si>
-  <si>
-    <t>Disco flap 4-1/2" grano 60 estricto gravado-7</t>
-  </si>
-  <si>
-    <t>Tornillo para concreto HUS3 M8 x 100 estricto gravado-8</t>
-  </si>
-  <si>
-    <t>Tornillo estructural para madera 8 x 2" estricto exonerado-9</t>
-  </si>
-  <si>
-    <t>Anclaje wedge Trubolt 5/8" x 6" estricto exonerado-10</t>
-  </si>
-  <si>
-    <t>Cartucho resina FIS V 300 ml estricto exonerado-11</t>
-  </si>
-  <si>
-    <t>Tubo PVC hidráulico 25 mm 6 m estricto exonerado-12</t>
-  </si>
-  <si>
-    <t>Tubería de cobre tipo L 3/4" estricto exonerado-13</t>
-  </si>
-  <si>
-    <t>Mezcladora lavabo monomando estricto inafecto-14</t>
-  </si>
-  <si>
-    <t>SikaTop Seal 5 impermeabilizante 4kg estricto inafecto-15</t>
-  </si>
-  <si>
-    <t>Llave ajustable 10" estricto gravado-5</t>
-  </si>
-  <si>
-    <t>Taladro percutor GSB 13 RE 1/2" estricto gravado-6</t>
-  </si>
-  <si>
-    <t>PRECIO ESTÁNDAR</t>
+    <t>Anclaje wedge Trubolt 5/8" x 6" flesible exonerado-8</t>
+  </si>
+  <si>
+    <t>Cartucho resina FIS V 300 ml flexible exonerado-9</t>
+  </si>
+  <si>
+    <t>Tubo PVC hidráulico 25 mm 6 m flexible exonerado-10</t>
+  </si>
+  <si>
+    <t>Tubería de cobre tipo L 3/4" flexible exonerado-11</t>
+  </si>
+  <si>
+    <t>Mezcladora lavabo monomando flexible inafecto-12</t>
+  </si>
+  <si>
+    <t>SikaTop Seal 5 impermeabilizante 4kg flexible inafecto-13</t>
   </si>
 </sst>
 </file>
@@ -1360,66 +1183,66 @@
   <sheetData>
     <row r="1" spans="1:12" s="6" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="9" t="s">
-        <v>7</v>
-      </c>
       <c r="I1" s="14" t="s">
-        <v>248</v>
+        <v>182</v>
       </c>
       <c r="J1" s="14" t="s">
-        <v>195</v>
+        <v>161</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>196</v>
+        <v>162</v>
       </c>
       <c r="L1" s="14" t="s">
-        <v>197</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>198</v>
+        <v>164</v>
       </c>
       <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" t="s">
         <v>113</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>114</v>
       </c>
-      <c r="D2" t="s">
-        <v>115</v>
-      </c>
       <c r="E2" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I2" s="15">
         <v>98.735399999999998</v>
@@ -1436,28 +1259,28 @@
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>199</v>
+        <v>165</v>
       </c>
       <c r="B3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D3" t="s">
         <v>116</v>
       </c>
-      <c r="C3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D3" t="s">
-        <v>117</v>
-      </c>
       <c r="E3" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I3" s="15">
         <v>193.6054</v>
@@ -1474,28 +1297,28 @@
     </row>
     <row r="4" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="B4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I4" s="15">
         <v>79.543300000000002</v>
@@ -1512,28 +1335,28 @@
     </row>
     <row r="5" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>201</v>
+        <v>167</v>
       </c>
       <c r="B5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" t="s">
         <v>119</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>120</v>
       </c>
-      <c r="D5" t="s">
-        <v>121</v>
-      </c>
       <c r="E5" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I5" s="15">
         <v>131.87190000000001</v>
@@ -1550,28 +1373,28 @@
     </row>
     <row r="6" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>207</v>
+        <v>172</v>
       </c>
       <c r="B6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" t="s">
         <v>122</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>123</v>
       </c>
-      <c r="D6" t="s">
-        <v>124</v>
-      </c>
       <c r="E6" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I6" s="15">
         <v>51.205100000000002</v>
@@ -1588,28 +1411,28 @@
     </row>
     <row r="7" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>208</v>
+        <v>173</v>
       </c>
       <c r="B7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" t="s">
         <v>125</v>
       </c>
-      <c r="C7" t="s">
-        <v>123</v>
-      </c>
-      <c r="D7" t="s">
-        <v>126</v>
-      </c>
       <c r="E7" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I7" s="15">
         <v>113.3768</v>
@@ -1626,28 +1449,28 @@
     </row>
     <row r="8" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>209</v>
+        <v>174</v>
       </c>
       <c r="B8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" t="s">
         <v>127</v>
       </c>
-      <c r="C8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" t="s">
-        <v>128</v>
-      </c>
       <c r="E8" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I8" s="15">
         <v>73.331100000000006</v>
@@ -1664,28 +1487,28 @@
     </row>
     <row r="9" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>210</v>
+        <v>175</v>
       </c>
       <c r="B9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" t="s">
         <v>129</v>
       </c>
-      <c r="C9" t="s">
-        <v>123</v>
-      </c>
-      <c r="D9" t="s">
-        <v>130</v>
-      </c>
       <c r="E9" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I9" s="15">
         <v>138.31399999999999</v>
@@ -1702,28 +1525,28 @@
     </row>
     <row r="10" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>211</v>
+        <v>176</v>
       </c>
       <c r="B10" t="s">
+        <v>130</v>
+      </c>
+      <c r="C10" t="s">
         <v>131</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>132</v>
       </c>
-      <c r="D10" t="s">
-        <v>133</v>
-      </c>
       <c r="E10" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I10" s="15">
         <v>39.536700000000003</v>
@@ -1740,28 +1563,28 @@
     </row>
     <row r="11" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>212</v>
+        <v>177</v>
       </c>
       <c r="B11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" t="s">
+        <v>131</v>
+      </c>
+      <c r="D11" t="s">
         <v>134</v>
       </c>
-      <c r="C11" t="s">
-        <v>132</v>
-      </c>
-      <c r="D11" t="s">
-        <v>135</v>
-      </c>
       <c r="E11" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I11" s="15">
         <v>132.9709</v>
@@ -1778,28 +1601,28 @@
     </row>
     <row r="12" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>213</v>
+        <v>178</v>
       </c>
       <c r="B12" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" t="s">
+        <v>131</v>
+      </c>
+      <c r="D12" t="s">
         <v>136</v>
       </c>
-      <c r="C12" t="s">
-        <v>132</v>
-      </c>
-      <c r="D12" t="s">
-        <v>137</v>
-      </c>
       <c r="E12" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I12" s="15">
         <v>29.781400000000001</v>
@@ -1816,28 +1639,28 @@
     </row>
     <row r="13" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>214</v>
+        <v>179</v>
       </c>
       <c r="B13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" t="s">
         <v>138</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>139</v>
       </c>
-      <c r="D13" t="s">
-        <v>140</v>
-      </c>
       <c r="E13" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I13" s="15">
         <v>25.97</v>
@@ -1854,28 +1677,28 @@
     </row>
     <row r="14" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>202</v>
+        <v>168</v>
       </c>
       <c r="B14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C14" t="s">
+        <v>138</v>
+      </c>
+      <c r="D14" t="s">
         <v>139</v>
       </c>
-      <c r="D14" t="s">
-        <v>140</v>
-      </c>
       <c r="E14" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I14" s="15">
         <v>115.6091</v>
@@ -1892,28 +1715,28 @@
     </row>
     <row r="15" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="B15" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" t="s">
         <v>142</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>143</v>
       </c>
-      <c r="D15" t="s">
-        <v>144</v>
-      </c>
       <c r="E15" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I15" s="15">
         <v>169.09280000000001</v>
@@ -1930,28 +1753,28 @@
     </row>
     <row r="16" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>204</v>
+        <v>170</v>
       </c>
       <c r="B16" t="s">
+        <v>144</v>
+      </c>
+      <c r="C16" t="s">
+        <v>142</v>
+      </c>
+      <c r="D16" t="s">
         <v>145</v>
       </c>
-      <c r="C16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D16" t="s">
-        <v>146</v>
-      </c>
       <c r="E16" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I16" s="15">
         <v>117.9316</v>
@@ -1968,28 +1791,28 @@
     </row>
     <row r="17" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>205</v>
+        <v>171</v>
       </c>
       <c r="B17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C17" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" t="s">
         <v>147</v>
       </c>
-      <c r="C17" t="s">
-        <v>143</v>
-      </c>
-      <c r="D17" t="s">
-        <v>148</v>
-      </c>
       <c r="E17" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I17" s="15">
         <v>65.521699999999996</v>
@@ -2006,28 +1829,28 @@
     </row>
     <row r="18" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>215</v>
+        <v>180</v>
       </c>
       <c r="B18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C18" t="s">
+        <v>142</v>
+      </c>
+      <c r="D18" t="s">
         <v>149</v>
       </c>
-      <c r="C18" t="s">
-        <v>143</v>
-      </c>
-      <c r="D18" t="s">
-        <v>150</v>
-      </c>
       <c r="E18" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I18" s="15">
         <v>3.5644</v>
@@ -2044,28 +1867,28 @@
     </row>
     <row r="19" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
-        <v>216</v>
+        <v>181</v>
       </c>
       <c r="B19" t="s">
+        <v>150</v>
+      </c>
+      <c r="C19" t="s">
         <v>151</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>152</v>
       </c>
-      <c r="D19" t="s">
-        <v>153</v>
-      </c>
       <c r="E19" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I19" s="15">
         <v>115.5861</v>
@@ -2082,28 +1905,28 @@
     </row>
     <row r="20" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>217</v>
+        <v>184</v>
       </c>
       <c r="B20" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C20" t="s">
+        <v>151</v>
+      </c>
+      <c r="D20" t="s">
         <v>152</v>
       </c>
-      <c r="D20" t="s">
-        <v>153</v>
-      </c>
       <c r="E20" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I20" s="15">
         <v>188.68600000000001</v>
@@ -2120,28 +1943,28 @@
     </row>
     <row r="21" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>218</v>
+        <v>185</v>
       </c>
       <c r="B21" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C21" t="s">
+        <v>154</v>
+      </c>
+      <c r="D21" t="s">
         <v>155</v>
       </c>
-      <c r="D21" t="s">
-        <v>156</v>
-      </c>
       <c r="E21" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I21" s="15">
         <v>48.632300000000001</v>
@@ -2158,28 +1981,28 @@
     </row>
     <row r="22" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>219</v>
+        <v>186</v>
       </c>
       <c r="B22" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C22" t="s">
+        <v>154</v>
+      </c>
+      <c r="D22" t="s">
         <v>155</v>
       </c>
-      <c r="D22" t="s">
-        <v>156</v>
-      </c>
       <c r="E22" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I22" s="15">
         <v>69.011899999999997</v>
@@ -2196,28 +2019,28 @@
     </row>
     <row r="23" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
-        <v>220</v>
+        <v>187</v>
       </c>
       <c r="B23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C23" t="s">
+        <v>154</v>
+      </c>
+      <c r="D23" t="s">
         <v>155</v>
       </c>
-      <c r="D23" t="s">
-        <v>156</v>
-      </c>
       <c r="E23" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I23" s="15">
         <v>112.0016</v>
@@ -2234,28 +2057,28 @@
     </row>
     <row r="24" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>221</v>
+        <v>188</v>
       </c>
       <c r="B24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
+        <v>158</v>
+      </c>
+      <c r="D24" t="s">
         <v>159</v>
       </c>
-      <c r="D24" t="s">
-        <v>160</v>
-      </c>
       <c r="E24" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I24" s="15">
         <v>182.41929999999999</v>
@@ -2272,28 +2095,28 @@
     </row>
     <row r="25" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>222</v>
+        <v>189</v>
       </c>
       <c r="B25" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C25" t="s">
+        <v>158</v>
+      </c>
+      <c r="D25" t="s">
         <v>159</v>
       </c>
-      <c r="D25" t="s">
-        <v>160</v>
-      </c>
       <c r="E25" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I25" s="15">
         <v>119.85380000000001</v>
@@ -2309,992 +2132,368 @@
       </c>
     </row>
     <row r="26" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="B26" t="s">
-        <v>162</v>
-      </c>
-      <c r="C26" t="s">
-        <v>159</v>
-      </c>
-      <c r="D26" t="s">
-        <v>160</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I26" s="15">
-        <v>40.133699999999997</v>
-      </c>
-      <c r="J26" s="15">
-        <v>34.113644999999998</v>
-      </c>
-      <c r="K26" s="15">
-        <v>11.337203389830508</v>
-      </c>
-      <c r="L26" s="15">
-        <v>26.086905000000002</v>
-      </c>
+      <c r="A26" s="7"/>
+      <c r="B26"/>
+      <c r="C26"/>
+      <c r="D26"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="15"/>
     </row>
     <row r="27" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="B27" t="s">
-        <v>163</v>
-      </c>
-      <c r="C27" t="s">
-        <v>159</v>
-      </c>
-      <c r="D27" t="s">
-        <v>160</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I27" s="15">
-        <v>103.6125</v>
-      </c>
-      <c r="J27" s="15">
-        <v>88.070624999999993</v>
-      </c>
-      <c r="K27" s="15">
-        <v>29.26906779661017</v>
-      </c>
-      <c r="L27" s="15">
-        <v>67.34812500000001</v>
-      </c>
+      <c r="A27" s="7"/>
+      <c r="B27"/>
+      <c r="C27"/>
+      <c r="D27"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="15"/>
+      <c r="L27" s="15"/>
     </row>
     <row r="28" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="B28" t="s">
-        <v>164</v>
-      </c>
-      <c r="C28" t="s">
-        <v>165</v>
-      </c>
-      <c r="D28" t="s">
-        <v>166</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I28" s="15">
-        <v>131.12729999999999</v>
-      </c>
-      <c r="J28" s="15">
-        <v>111.45820499999999</v>
-      </c>
-      <c r="K28" s="15">
-        <v>37.04161016949152</v>
-      </c>
-      <c r="L28" s="15">
-        <v>85.232744999999994</v>
-      </c>
+      <c r="A28" s="7"/>
+      <c r="B28"/>
+      <c r="C28"/>
+      <c r="D28"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="15"/>
     </row>
     <row r="29" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="B29" t="s">
-        <v>167</v>
-      </c>
-      <c r="C29" t="s">
-        <v>165</v>
-      </c>
-      <c r="D29" t="s">
-        <v>166</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I29" s="15">
-        <v>6.5842999999999998</v>
-      </c>
-      <c r="J29" s="15">
-        <v>5.5966550000000002</v>
-      </c>
-      <c r="K29" s="15">
-        <v>1.8599717514124292</v>
-      </c>
-      <c r="L29" s="15">
-        <v>4.279795</v>
-      </c>
+      <c r="A29" s="7"/>
+      <c r="B29"/>
+      <c r="C29"/>
+      <c r="D29"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="15"/>
     </row>
     <row r="30" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="B30" t="s">
-        <v>168</v>
-      </c>
-      <c r="C30" t="s">
-        <v>169</v>
-      </c>
-      <c r="D30" t="s">
-        <v>170</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I30" s="15">
-        <v>7.2276999999999996</v>
-      </c>
-      <c r="J30" s="15">
-        <v>6.1435449999999996</v>
-      </c>
-      <c r="K30" s="15">
-        <v>2.0417231638418079</v>
-      </c>
-      <c r="L30" s="15">
-        <v>4.6980050000000002</v>
-      </c>
+      <c r="A30" s="7"/>
+      <c r="B30"/>
+      <c r="C30"/>
+      <c r="D30"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="15"/>
+      <c r="L30" s="15"/>
     </row>
     <row r="31" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="B31" t="s">
-        <v>171</v>
-      </c>
-      <c r="C31" t="s">
-        <v>169</v>
-      </c>
-      <c r="D31" t="s">
-        <v>170</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I31" s="15">
-        <v>94.335499999999996</v>
-      </c>
-      <c r="J31" s="15">
-        <v>80.185175000000001</v>
-      </c>
-      <c r="K31" s="15">
-        <v>26.648446327683615</v>
-      </c>
-      <c r="L31" s="15">
-        <v>61.318075</v>
-      </c>
+      <c r="A31" s="7"/>
+      <c r="B31"/>
+      <c r="C31"/>
+      <c r="D31"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="15"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="15"/>
     </row>
     <row r="32" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="B32" t="s">
-        <v>172</v>
-      </c>
-      <c r="C32" t="s">
-        <v>173</v>
-      </c>
-      <c r="D32" t="s">
-        <v>174</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I32" s="15">
-        <v>14.8171</v>
-      </c>
-      <c r="J32" s="15">
-        <v>12.594535</v>
-      </c>
-      <c r="K32" s="15">
-        <v>4.1856214689265538</v>
-      </c>
-      <c r="L32" s="15">
-        <v>9.6311150000000012</v>
-      </c>
+      <c r="A32" s="7"/>
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
     </row>
     <row r="33" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="B33" t="s">
-        <v>175</v>
-      </c>
-      <c r="C33" t="s">
-        <v>173</v>
-      </c>
-      <c r="D33" t="s">
-        <v>174</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I33" s="15">
-        <v>61.024000000000001</v>
-      </c>
-      <c r="J33" s="15">
-        <v>51.870400000000004</v>
-      </c>
-      <c r="K33" s="15">
-        <v>17.238418079096046</v>
-      </c>
-      <c r="L33" s="15">
-        <v>39.665599999999998</v>
-      </c>
+      <c r="A33" s="7"/>
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="15"/>
     </row>
     <row r="34" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="B34" t="s">
-        <v>176</v>
-      </c>
-      <c r="C34" t="s">
-        <v>177</v>
-      </c>
-      <c r="D34" t="s">
-        <v>178</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G34" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I34" s="15">
-        <v>3.9333</v>
-      </c>
-      <c r="J34" s="15">
-        <v>3.343305</v>
-      </c>
-      <c r="K34" s="15">
-        <v>1.1111016949152541</v>
-      </c>
-      <c r="L34" s="15">
-        <v>2.5566450000000001</v>
-      </c>
+      <c r="A34" s="7"/>
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
     </row>
     <row r="35" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="B35" t="s">
-        <v>179</v>
-      </c>
-      <c r="C35" t="s">
-        <v>177</v>
-      </c>
-      <c r="D35" t="s">
-        <v>178</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I35" s="15">
-        <v>63.429299999999998</v>
-      </c>
-      <c r="J35" s="15">
-        <v>53.914904999999997</v>
-      </c>
-      <c r="K35" s="15">
-        <v>17.917881355932202</v>
-      </c>
-      <c r="L35" s="15">
-        <v>41.229044999999999</v>
-      </c>
+      <c r="A35" s="7"/>
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
     </row>
     <row r="36" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="B36" t="s">
-        <v>180</v>
-      </c>
-      <c r="C36" t="s">
-        <v>177</v>
-      </c>
-      <c r="D36" t="s">
-        <v>178</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G36" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I36" s="15">
-        <v>125.7509</v>
-      </c>
-      <c r="J36" s="15">
-        <v>106.888265</v>
-      </c>
-      <c r="K36" s="15">
-        <v>35.522853107344631</v>
-      </c>
-      <c r="L36" s="15">
-        <v>81.738085000000012</v>
-      </c>
+      <c r="A36" s="7"/>
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
+      <c r="K36" s="15"/>
+      <c r="L36" s="15"/>
     </row>
     <row r="37" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="B37" t="s">
-        <v>181</v>
-      </c>
-      <c r="C37" t="s">
-        <v>177</v>
-      </c>
-      <c r="D37" t="s">
-        <v>182</v>
-      </c>
-      <c r="E37" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="I37" s="15">
-        <v>79.836799999999997</v>
-      </c>
-      <c r="J37" s="15">
-        <v>67.861279999999994</v>
-      </c>
-      <c r="K37" s="15">
-        <v>22.552768361581919</v>
-      </c>
-      <c r="L37" s="15">
-        <v>51.893919999999994</v>
-      </c>
+      <c r="A37" s="7"/>
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="15"/>
+      <c r="J37" s="15"/>
+      <c r="K37" s="15"/>
+      <c r="L37" s="15"/>
     </row>
     <row r="38" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="B38" t="s">
-        <v>181</v>
-      </c>
-      <c r="C38" t="s">
-        <v>177</v>
-      </c>
-      <c r="D38" t="s">
-        <v>182</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G38" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I38" s="15">
-        <v>156.43209999999999</v>
-      </c>
-      <c r="J38" s="15">
-        <v>132.967285</v>
-      </c>
-      <c r="K38" s="15">
-        <v>44.189858757062147</v>
-      </c>
-      <c r="L38" s="15">
-        <v>101.680865</v>
-      </c>
+      <c r="A38" s="7"/>
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15"/>
+      <c r="L38" s="15"/>
     </row>
     <row r="39" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="B39" t="s">
-        <v>172</v>
-      </c>
-      <c r="C39" t="s">
-        <v>183</v>
-      </c>
-      <c r="D39" t="s">
-        <v>184</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I39" s="15">
-        <v>169.0153</v>
-      </c>
-      <c r="J39" s="15">
-        <v>143.663005</v>
-      </c>
-      <c r="K39" s="15">
-        <v>47.744435028248589</v>
-      </c>
-      <c r="L39" s="15">
-        <v>109.85994500000001</v>
-      </c>
+      <c r="A39" s="7"/>
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="15"/>
+      <c r="K39" s="15"/>
+      <c r="L39" s="15"/>
     </row>
     <row r="40" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="B40" t="s">
-        <v>185</v>
-      </c>
-      <c r="C40" t="s">
-        <v>183</v>
-      </c>
-      <c r="D40" t="s">
-        <v>184</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G40" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I40" s="15">
-        <v>166.46690000000001</v>
-      </c>
-      <c r="J40" s="15">
-        <v>141.49686500000001</v>
-      </c>
-      <c r="K40" s="15">
-        <v>47.024548022598871</v>
-      </c>
-      <c r="L40" s="15">
-        <v>108.203485</v>
-      </c>
+      <c r="A40" s="7"/>
+      <c r="B40"/>
+      <c r="C40"/>
+      <c r="D40"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15"/>
+      <c r="L40" s="15"/>
     </row>
     <row r="41" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="B41" t="s">
-        <v>113</v>
-      </c>
-      <c r="C41" t="s">
-        <v>186</v>
-      </c>
-      <c r="D41" t="s">
-        <v>187</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I41" s="15">
-        <v>108.5399</v>
-      </c>
-      <c r="J41" s="15">
-        <v>92.258915000000002</v>
-      </c>
-      <c r="K41" s="15">
-        <v>30.660988700564971</v>
-      </c>
-      <c r="L41" s="15">
-        <v>70.55093500000001</v>
-      </c>
+      <c r="A41" s="7"/>
+      <c r="B41"/>
+      <c r="C41"/>
+      <c r="D41"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="15"/>
+      <c r="L41" s="15"/>
     </row>
     <row r="42" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="B42" t="s">
-        <v>113</v>
-      </c>
-      <c r="C42" t="s">
-        <v>186</v>
-      </c>
-      <c r="D42" t="s">
-        <v>187</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G42" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I42" s="15">
-        <v>51.077800000000003</v>
-      </c>
-      <c r="J42" s="15">
-        <v>43.416130000000003</v>
-      </c>
-      <c r="K42" s="15">
-        <v>14.428757062146893</v>
-      </c>
-      <c r="L42" s="15">
-        <v>33.200569999999999</v>
-      </c>
+      <c r="A42" s="7"/>
+      <c r="B42"/>
+      <c r="C42"/>
+      <c r="D42"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="15"/>
+      <c r="J42" s="15"/>
+      <c r="K42" s="15"/>
+      <c r="L42" s="15"/>
     </row>
     <row r="43" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="B43" t="s">
-        <v>188</v>
-      </c>
-      <c r="C43" t="s">
-        <v>143</v>
-      </c>
-      <c r="D43" t="s">
-        <v>148</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G43" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="I43" s="15">
-        <v>124.13079999999999</v>
-      </c>
-      <c r="J43" s="15">
-        <v>105.51118</v>
-      </c>
-      <c r="K43" s="15">
-        <v>35.065197740112993</v>
-      </c>
-      <c r="L43" s="15">
-        <v>80.685020000000009</v>
-      </c>
+      <c r="A43" s="7"/>
+      <c r="B43"/>
+      <c r="C43"/>
+      <c r="D43"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="15"/>
+      <c r="J43" s="15"/>
+      <c r="K43" s="15"/>
+      <c r="L43" s="15"/>
     </row>
     <row r="44" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="B44" t="s">
-        <v>189</v>
-      </c>
-      <c r="C44" t="s">
-        <v>143</v>
-      </c>
-      <c r="D44" t="s">
-        <v>148</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I44" s="15">
-        <v>67.139200000000002</v>
-      </c>
-      <c r="J44" s="15">
-        <v>57.06832</v>
-      </c>
-      <c r="K44" s="15">
-        <v>18.965875706214689</v>
-      </c>
-      <c r="L44" s="15">
-        <v>43.640480000000004</v>
-      </c>
+      <c r="A44" s="7"/>
+      <c r="B44"/>
+      <c r="C44"/>
+      <c r="D44"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
+      <c r="H44" s="7"/>
+      <c r="I44" s="15"/>
+      <c r="J44" s="15"/>
+      <c r="K44" s="15"/>
+      <c r="L44" s="15"/>
     </row>
     <row r="45" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="B45" t="s">
-        <v>190</v>
-      </c>
-      <c r="C45" t="s">
-        <v>143</v>
-      </c>
-      <c r="D45" t="s">
-        <v>148</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G45" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I45" s="15">
-        <v>95.355900000000005</v>
-      </c>
-      <c r="J45" s="15">
-        <v>81.052515</v>
-      </c>
-      <c r="K45" s="15">
-        <v>26.93669491525424</v>
-      </c>
-      <c r="L45" s="15">
-        <v>61.981335000000009</v>
-      </c>
+      <c r="A45" s="7"/>
+      <c r="B45"/>
+      <c r="C45"/>
+      <c r="D45"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="15"/>
+      <c r="J45" s="15"/>
+      <c r="K45" s="15"/>
+      <c r="L45" s="15"/>
     </row>
     <row r="46" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="B46" t="s">
-        <v>141</v>
-      </c>
-      <c r="C46" t="s">
-        <v>139</v>
-      </c>
-      <c r="D46" t="s">
-        <v>140</v>
-      </c>
-      <c r="E46" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F46" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G46" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I46" s="15">
-        <v>100.6953</v>
-      </c>
-      <c r="J46" s="15">
-        <v>85.591004999999996</v>
-      </c>
-      <c r="K46" s="15">
-        <v>28.445</v>
-      </c>
-      <c r="L46" s="15">
-        <v>65.451944999999995</v>
-      </c>
+      <c r="A46" s="7"/>
+      <c r="B46"/>
+      <c r="C46"/>
+      <c r="D46"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
+      <c r="K46" s="15"/>
+      <c r="L46" s="15"/>
     </row>
     <row r="47" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="B47" t="s">
-        <v>190</v>
-      </c>
-      <c r="C47" t="s">
-        <v>143</v>
-      </c>
-      <c r="D47" t="s">
-        <v>148</v>
-      </c>
-      <c r="E47" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G47" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I47" s="15">
-        <v>95.4392</v>
-      </c>
-      <c r="J47" s="15">
-        <v>81.123320000000007</v>
-      </c>
-      <c r="K47" s="15">
-        <v>26.960225988700564</v>
-      </c>
-      <c r="L47" s="15">
-        <v>62.03548</v>
-      </c>
+      <c r="A47" s="7"/>
+      <c r="B47"/>
+      <c r="C47"/>
+      <c r="D47"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15"/>
+      <c r="K47" s="15"/>
+      <c r="L47" s="15"/>
     </row>
     <row r="48" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="B48" t="s">
-        <v>191</v>
-      </c>
-      <c r="C48" t="s">
-        <v>114</v>
-      </c>
-      <c r="D48" t="s">
-        <v>115</v>
-      </c>
-      <c r="E48" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F48" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I48" s="15">
-        <v>182.11840000000001</v>
-      </c>
-      <c r="J48" s="15">
-        <v>154.80064000000002</v>
-      </c>
-      <c r="K48" s="15">
-        <v>51.445875706214693</v>
-      </c>
-      <c r="L48" s="15">
-        <v>118.37696000000001</v>
-      </c>
+      <c r="A48" s="7"/>
+      <c r="B48"/>
+      <c r="C48"/>
+      <c r="D48"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
     </row>
     <row r="49" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="B49" t="s">
-        <v>192</v>
-      </c>
-      <c r="C49" t="s">
-        <v>114</v>
-      </c>
-      <c r="D49" t="s">
-        <v>117</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F49" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G49" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I49" s="15">
-        <v>171.61009999999999</v>
-      </c>
-      <c r="J49" s="15">
-        <v>145.868585</v>
-      </c>
-      <c r="K49" s="15">
-        <v>48.47742937853107</v>
-      </c>
-      <c r="L49" s="15">
-        <v>111.54656499999999</v>
-      </c>
+      <c r="A49" s="7"/>
+      <c r="B49"/>
+      <c r="C49"/>
+      <c r="D49"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="15"/>
+      <c r="J49" s="15"/>
+      <c r="K49" s="15"/>
+      <c r="L49" s="15"/>
     </row>
     <row r="50" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="B50" t="s">
-        <v>193</v>
-      </c>
-      <c r="C50" t="s">
-        <v>114</v>
-      </c>
-      <c r="D50" t="s">
-        <v>117</v>
-      </c>
-      <c r="E50" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I50" s="15">
-        <v>3.2168999999999999</v>
-      </c>
-      <c r="J50" s="15">
-        <v>2.7343649999999999</v>
-      </c>
-      <c r="K50" s="15">
-        <v>0.908728813559322</v>
-      </c>
-      <c r="L50" s="15">
-        <v>2.0909849999999999</v>
-      </c>
+      <c r="A50" s="7"/>
+      <c r="B50"/>
+      <c r="C50"/>
+      <c r="D50"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="15"/>
+      <c r="J50" s="15"/>
+      <c r="K50" s="15"/>
+      <c r="L50" s="15"/>
     </row>
     <row r="51" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="B51" t="s">
-        <v>194</v>
-      </c>
-      <c r="C51" t="s">
-        <v>152</v>
-      </c>
-      <c r="D51" t="s">
-        <v>153</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="I51" s="15">
-        <v>131.45660000000001</v>
-      </c>
-      <c r="J51" s="15">
-        <v>111.73811000000001</v>
-      </c>
-      <c r="K51" s="15">
-        <v>37.134632768361584</v>
-      </c>
-      <c r="L51" s="15">
-        <v>85.446790000000007</v>
-      </c>
+      <c r="A51" s="7"/>
+      <c r="B51"/>
+      <c r="C51"/>
+      <c r="D51"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="15"/>
+      <c r="J51" s="15"/>
+      <c r="K51" s="15"/>
+      <c r="L51" s="15"/>
     </row>
     <row r="52" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="7"/>
@@ -4439,542 +3638,542 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B20" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B28" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B31" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B32" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B37" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B38" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B39" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B40" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B41" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B42" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B43" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="47" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B48" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B49" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B50" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B51" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B52" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B56" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B57" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="58" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B58" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="59" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B59" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="60" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B60" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="61" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B61" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="62" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B62" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B63" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B64" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B65" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B66" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B67" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B68" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B69" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B70" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B71" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B72" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="73" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B73" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B74" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B75" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B76" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B77" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B78" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B79" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B80" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B81" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B82" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B83" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="84" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B84" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B85" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B86" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B87" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B88" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B89" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="90" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B90" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B91" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B92" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B93" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B94" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="95" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B95" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B96" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B97" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B98" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B99" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B100" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B101" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B102" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="103" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B103" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B104" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B105" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="106" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B106" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B107" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B108" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="109" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B109" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B110" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B111" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B112" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B113" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="114" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B114" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B115" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B116" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="117" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B117" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="120" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B120" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B121" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="122" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B122" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="123" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B123" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cambiando cabecera columna de productos de Descripcion -> NOMBRE
</commit_message>
<xml_diff>
--- a/src/data/FORMATO_SUBIDA_PRODUCTOS.xlsx
+++ b/src/data/FORMATO_SUBIDA_PRODUCTOS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WebstormProjects\erpperu2-automation\src\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WebstormProjects\erpperu2-automation-main\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B6BA12-DD08-4B1D-B6C6-BA08DEF66E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6180DB65-880C-441C-8FAD-E8E4FB70F330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31185" yWindow="3315" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCTOS" sheetId="1" r:id="rId1"/>
@@ -581,9 +581,6 @@
     <t>PRECIO ESTÁNDAR</t>
   </si>
   <si>
-    <t>DESCRIPCION</t>
-  </si>
-  <si>
     <t>Anclaje wedge Trubolt 5/8" x 6" flesible exonerado-8</t>
   </si>
   <si>
@@ -600,6 +597,9 @@
   </si>
   <si>
     <t>SikaTop Seal 5 impermeabilizante 4kg flexible inafecto-13</t>
+  </si>
+  <si>
+    <t>NOMBRE</t>
   </si>
 </sst>
 </file>
@@ -609,7 +609,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -657,6 +657,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -831,7 +839,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -862,6 +870,7 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1183,7 +1192,7 @@
   <sheetData>
     <row r="1" spans="1:12" s="6" customFormat="1" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
@@ -1258,7 +1267,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="16" t="s">
         <v>165</v>
       </c>
       <c r="B3" t="s">
@@ -1905,7 +1914,7 @@
     </row>
     <row r="20" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B20" t="s">
         <v>153</v>
@@ -1943,7 +1952,7 @@
     </row>
     <row r="21" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B21" t="s">
         <v>140</v>
@@ -1981,7 +1990,7 @@
     </row>
     <row r="22" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B22" t="s">
         <v>156</v>
@@ -2019,7 +2028,7 @@
     </row>
     <row r="23" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B23" t="s">
         <v>157</v>
@@ -2057,7 +2066,7 @@
     </row>
     <row r="24" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B24" t="s">
         <v>112</v>
@@ -2095,7 +2104,7 @@
     </row>
     <row r="25" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B25" t="s">
         <v>160</v>

</xml_diff>